<commit_message>
feilds removed in price list
</commit_message>
<xml_diff>
--- a/public/templates/Crackers_90_Percent_PriceList_Template.xlsx
+++ b/public/templates/Crackers_90_Percent_PriceList_Template.xlsx
@@ -397,17 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:F7"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="36.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -427,16 +424,7 @@
         <v>MRP Price / Rate</v>
       </c>
       <c r="F1" t="str">
-        <v>90% Discount</v>
-      </c>
-      <c r="G1" t="str">
         <v>Per / PCS</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Net Rate</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Stock</v>
       </c>
     </row>
     <row r="2">
@@ -455,17 +443,8 @@
       <c r="E2">
         <v>100</v>
       </c>
-      <c r="F2">
-        <v>90</v>
-      </c>
-      <c r="G2" t="str">
+      <c r="F2" t="str">
         <v>Box</v>
-      </c>
-      <c r="H2">
-        <v>10</v>
-      </c>
-      <c r="I2">
-        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -484,17 +463,8 @@
       <c r="E3">
         <v>200</v>
       </c>
-      <c r="F3">
-        <v>90</v>
-      </c>
-      <c r="G3" t="str">
+      <c r="F3" t="str">
         <v>Box</v>
-      </c>
-      <c r="H3">
-        <v>20</v>
-      </c>
-      <c r="I3">
-        <v>400</v>
       </c>
     </row>
     <row r="4">
@@ -513,17 +483,8 @@
       <c r="E4">
         <v>80</v>
       </c>
-      <c r="F4">
-        <v>90</v>
-      </c>
-      <c r="G4" t="str">
+      <c r="F4" t="str">
         <v>Box</v>
-      </c>
-      <c r="H4">
-        <v>8</v>
-      </c>
-      <c r="I4">
-        <v>600</v>
       </c>
     </row>
     <row r="5">
@@ -542,17 +503,8 @@
       <c r="E5">
         <v>450</v>
       </c>
-      <c r="F5">
-        <v>90</v>
-      </c>
-      <c r="G5" t="str">
+      <c r="F5" t="str">
         <v>Box</v>
-      </c>
-      <c r="H5">
-        <v>45</v>
-      </c>
-      <c r="I5">
-        <v>200</v>
       </c>
     </row>
     <row r="6">
@@ -571,17 +523,8 @@
       <c r="E6">
         <v>900</v>
       </c>
-      <c r="F6">
-        <v>90</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="F6" t="str">
         <v>Box</v>
-      </c>
-      <c r="H6">
-        <v>90</v>
-      </c>
-      <c r="I6">
-        <v>150</v>
       </c>
     </row>
     <row r="7">
@@ -600,22 +543,13 @@
       <c r="E7">
         <v>140</v>
       </c>
-      <c r="F7">
-        <v>90</v>
-      </c>
-      <c r="G7" t="str">
+      <c r="F7" t="str">
         <v>Box</v>
-      </c>
-      <c r="H7">
-        <v>14</v>
-      </c>
-      <c r="I7">
-        <v>250</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>